<commit_message>
v1.2.0: fixed source list with spend-channel rollup, exit strategy and disposition on every property
Sources: PPC, TV, SEO, Motivated Leads, DM Postcard, DM Letters, DM Checks,
Realtor, Other. REI BlackBook and whiteboard spellings normalize on paste and
edit. Each source rolls into one of six spend channels (adds SEO and Direct
mail to the day log) so cost per lead is per channel; Marketing dashboard
lists leads by source.

Exit strategy (Wholesale, Wholetail, Fix & Flip, Wholetail / Flip, Hold) and
disposition (Under construction, Listed, Listed - pending, Sold, Wholesaled)
live in the drawer under Deal; disposition shows on the Closed tab.

New columns append to existing sheets by re-running setupDatabase (tested).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PD4vD51siFq5jYyNjR6B3w
</commit_message>
<xml_diff>
--- a/apps/acquisitions-desk/docs/THB_Acquisitions_Desk_Production_Database_TEMPLATE.xlsx
+++ b/apps/acquisitions-desk/docs/THB_Acquisitions_Desk_Production_Database_TEMPLATE.xlsx
@@ -534,12 +534,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -579,12 +579,12 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -624,12 +624,12 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -665,12 +665,12 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -706,12 +706,12 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -747,12 +747,12 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -788,12 +788,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -829,12 +829,12 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -870,12 +870,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -911,12 +911,12 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA2"/>
+  <dimension ref="A1:AC2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1182,6 +1182,8 @@
     <col width="14" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="14" customWidth="1" min="27" max="27"/>
+    <col width="17" customWidth="1" min="28" max="28"/>
+    <col width="15" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1318,6 +1320,16 @@
       <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>version</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>exit_strategy</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>disposition</t>
         </is>
       </c>
     </row>
@@ -1349,6 +1361,8 @@
       <c r="Y2" s="2" t="n"/>
       <c r="Z2" s="2" t="n"/>
       <c r="AA2" s="2" t="n"/>
+      <c r="AB2" s="2" t="n"/>
+      <c r="AC2" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1576,7 +1590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1597,6 +1611,8 @@
     <col width="14" customWidth="1" min="16" max="16"/>
     <col width="14" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1688,6 +1704,16 @@
       <c r="R1" s="1" t="inlineStr">
         <is>
           <t>updated_at</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>seo_spend</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>mail_spend</t>
         </is>
       </c>
     </row>
@@ -1710,6 +1736,8 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1888,12 +1916,12 @@
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -1948,12 +1976,12 @@
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -2012,12 +2040,12 @@
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -2076,12 +2104,12 @@
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -2136,12 +2164,12 @@
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -2196,12 +2224,12 @@
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -2256,12 +2284,12 @@
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -2316,12 +2344,12 @@
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -2376,12 +2404,12 @@
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -2436,12 +2464,12 @@
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -2496,12 +2524,12 @@
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -2556,12 +2584,12 @@
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -2616,12 +2644,12 @@
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -2676,12 +2704,12 @@
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="R15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -2736,12 +2764,12 @@
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="R16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -2796,12 +2824,12 @@
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="R17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -2856,12 +2884,12 @@
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="R18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -2916,12 +2944,12 @@
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -2976,12 +3004,12 @@
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="R20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -3036,12 +3064,12 @@
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="R21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -3096,12 +3124,12 @@
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="R22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -3156,12 +3184,12 @@
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
       <c r="R23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -3321,7 +3349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -3370,7 +3398,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -3392,7 +3420,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -3414,7 +3442,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -3436,7 +3464,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -3458,7 +3486,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -3480,7 +3508,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -3492,7 +3520,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>1.0.0</t>
+          <t>1.2.0</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -3502,7 +3530,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -3524,7 +3552,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>
@@ -3546,7 +3574,51 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T19:33:51.000Z</t>
+          <t>2026-09-11T23:41:19.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>cpl_ceiling</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM_SETUP</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11T23:41:19.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>speed_target_minutes</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM_SETUP</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11T23:41:19.000Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v1.3.1: the rest of the team, one entry per person, real dates on tool handover
Adds the thirteen people from the PC board who were missing: Genesis, Gian,
Lawrence, Christine Joy, Mc, Jesery, Arjane, John, Kristine, Denzel, Darlyn,
Leo and Marieflor. No emails invented, so each is inactive until an admin sets
one; everyone new starts as TECHNICAL, which cannot work properties.

Re-running setupDatabase now tops up missing people instead of skipping once
the table has rows, and never edits a row that already exists, so a role, team
or email set by hand survives and a deactivated person stays deactivated.

A duplicate name is refused on creation, and a tool's trained list shows one
chip per person, keeping the entry that can sign in.

Asked builder for steps and Handed to the user on are date pickers, validated
as dates rather than stored as free text.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PD4vD51siFq5jYyNjR6B3w
</commit_message>
<xml_diff>
--- a/apps/acquisitions-desk/docs/THB_Acquisitions_Desk_Production_Database_TEMPLATE.xlsx
+++ b/apps/acquisitions-desk/docs/THB_Acquisitions_Desk_Production_Database_TEMPLATE.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -534,12 +534,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -579,12 +579,12 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -624,12 +624,12 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -665,12 +665,12 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -706,12 +706,12 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -747,12 +747,12 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -788,12 +788,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -829,12 +829,12 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -870,12 +870,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -911,12 +911,545 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>USR-GENESIS</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Genesis</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Acquisitions</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>REP</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>USR-GIAN</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Gian</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>AI &amp; Systems</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>TECHNICAL</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>USR-LAWRENCE</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Lawrence</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>AI &amp; Systems</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>TECHNICAL</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>USR-CHRISTINE</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Christine Joy</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>AI &amp; Systems</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>TECHNICAL</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>USR-MC</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Mc</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>AI &amp; Systems</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>TECHNICAL</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>USR-JESERY</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Jesery</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr"/>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>TECHNICAL</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>USR-ARJANE</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Arjane</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>TECHNICAL</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>USR-JOHN</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>John</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr"/>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>TECHNICAL</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>USR-KRISTINE</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Kristine</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>TECHNICAL</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>USR-DENZEL</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Denzel</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr"/>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>TECHNICAL</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>USR-DARLYN</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Darlyn</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>TECHNICAL</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>USR-LEO</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Leo</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr"/>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>TECHNICAL</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>USR-MARIEFLOR</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Marieflor</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>TECHNICAL</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -1923,12 +2456,12 @@
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -1983,12 +2516,12 @@
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -2047,12 +2580,12 @@
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -2111,12 +2644,12 @@
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -2171,12 +2704,12 @@
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -2231,12 +2764,12 @@
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -2291,12 +2824,12 @@
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -2351,12 +2884,12 @@
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -2411,12 +2944,12 @@
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -2471,12 +3004,12 @@
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -2531,12 +3064,12 @@
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -2591,12 +3124,12 @@
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -2651,12 +3184,12 @@
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -2711,12 +3244,12 @@
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="R15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -2771,12 +3304,12 @@
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="R16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -2831,12 +3364,12 @@
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="R17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -2891,12 +3424,12 @@
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="R18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -2951,12 +3484,12 @@
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -3011,12 +3544,12 @@
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="R20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -3071,12 +3604,12 @@
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="R21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -3131,12 +3664,12 @@
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="R22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -3191,12 +3724,12 @@
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
       <c r="R23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -3405,7 +3938,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -3427,7 +3960,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -3449,7 +3982,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -3471,7 +4004,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -3493,7 +4026,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -3515,7 +4048,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -3527,7 +4060,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>1.3.0</t>
+          <t>1.3.1</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -3537,7 +4070,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -3559,7 +4092,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -3581,7 +4114,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -3603,7 +4136,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>
@@ -3625,7 +4158,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:13:56.000Z</t>
+          <t>2026-09-12T16:41:23.000Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v1.4.0: closing date and sale price, and the whiteboard as a reviewable one-time update
Every property gains a closing date and a sale price next to the purchase
price. A sold property shows its sale price on the Closed tab row.

Whiteboard.gs transcribes the office board photographed 2026-09-12.
previewWhiteboardUpdate reports what would change and writes nothing;
applyWhiteboardUpdate writes through the normal lead API, so each change is
version checked, logged and attributed. Matching is by a distinctive part of
the address, and a row that matches nothing or several properties is reported
and skipped rather than guessed at. Running it twice changes nothing.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PD4vD51siFq5jYyNjR6B3w
</commit_message>
<xml_diff>
--- a/apps/acquisitions-desk/docs/THB_Acquisitions_Desk_Production_Database_TEMPLATE.xlsx
+++ b/apps/acquisitions-desk/docs/THB_Acquisitions_Desk_Production_Database_TEMPLATE.xlsx
@@ -534,12 +534,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -579,12 +579,12 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -624,12 +624,12 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -665,12 +665,12 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -706,12 +706,12 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -747,12 +747,12 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -788,12 +788,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -829,12 +829,12 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -870,12 +870,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -911,12 +911,12 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -952,12 +952,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -993,12 +993,12 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -1034,12 +1034,12 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -1075,12 +1075,12 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -1116,12 +1116,12 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -1157,12 +1157,12 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -1198,12 +1198,12 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -1239,12 +1239,12 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -1280,12 +1280,12 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -1321,12 +1321,12 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -1403,12 +1403,12 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -1444,12 +1444,12 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -1685,7 +1685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD2"/>
+  <dimension ref="A1:AF2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1718,6 +1718,8 @@
     <col width="17" customWidth="1" min="28" max="28"/>
     <col width="15" customWidth="1" min="29" max="29"/>
     <col width="18" customWidth="1" min="30" max="30"/>
+    <col width="16" customWidth="1" min="31" max="31"/>
+    <col width="14" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1869,6 +1871,16 @@
       <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>purchase_price</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>closing_date</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>sale_price</t>
         </is>
       </c>
     </row>
@@ -1903,6 +1915,8 @@
       <c r="AB2" s="2" t="n"/>
       <c r="AC2" s="2" t="n"/>
       <c r="AD2" s="2" t="n"/>
+      <c r="AE2" s="2" t="n"/>
+      <c r="AF2" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2456,12 +2470,12 @@
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -2516,12 +2530,12 @@
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -2580,12 +2594,12 @@
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -2644,12 +2658,12 @@
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -2704,12 +2718,12 @@
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -2764,12 +2778,12 @@
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -2824,12 +2838,12 @@
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -2884,12 +2898,12 @@
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -2944,12 +2958,12 @@
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -3004,12 +3018,12 @@
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -3064,12 +3078,12 @@
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -3124,12 +3138,12 @@
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -3184,12 +3198,12 @@
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -3244,12 +3258,12 @@
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="R15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -3304,12 +3318,12 @@
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="R16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -3364,12 +3378,12 @@
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="R17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -3424,12 +3438,12 @@
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="R18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -3484,12 +3498,12 @@
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -3544,12 +3558,12 @@
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="R20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -3604,12 +3618,12 @@
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="R21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -3664,12 +3678,12 @@
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="R22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -3724,12 +3738,12 @@
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
       <c r="R23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -3938,7 +3952,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -3960,7 +3974,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -3982,7 +3996,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -4004,7 +4018,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -4026,7 +4040,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -4048,7 +4062,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -4060,7 +4074,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>1.3.1</t>
+          <t>1.4.0</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -4070,7 +4084,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -4092,7 +4106,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -4114,7 +4128,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -4136,7 +4150,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>
@@ -4158,7 +4172,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T16:41:23.000Z</t>
+          <t>2026-09-12T17:03:53.000Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v1.5.0: seller email field, and a pass that takes the REI BlackBook tags out of the notes
Imported properties carried their REI BlackBook tag list in the Background
note. Those tags repeat the status and the source, and after the whiteboard
run some of them contradicted the source outright.

TidyNotes.gs reads a note as a list of fragments: an email moves into the new
seller_email field rather than being lost, a known tag is dropped, and
anything else is kept because a person wrote it. previewTidyNotes reports
without writing; applyTidyNotes writes through the normal lead API and is a
no-op on a second run.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PD4vD51siFq5jYyNjR6B3w
</commit_message>
<xml_diff>
--- a/apps/acquisitions-desk/docs/THB_Acquisitions_Desk_Production_Database_TEMPLATE.xlsx
+++ b/apps/acquisitions-desk/docs/THB_Acquisitions_Desk_Production_Database_TEMPLATE.xlsx
@@ -534,12 +534,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -579,12 +579,12 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -624,12 +624,12 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -665,12 +665,12 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -706,12 +706,12 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -747,12 +747,12 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -788,12 +788,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -829,12 +829,12 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -870,12 +870,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -911,12 +911,12 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -952,12 +952,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -993,12 +993,12 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -1034,12 +1034,12 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -1075,12 +1075,12 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -1116,12 +1116,12 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -1157,12 +1157,12 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -1198,12 +1198,12 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -1239,12 +1239,12 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -1280,12 +1280,12 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -1321,12 +1321,12 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -1403,12 +1403,12 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -1444,12 +1444,12 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -1685,7 +1685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF2"/>
+  <dimension ref="A1:AG2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1720,6 +1720,7 @@
     <col width="18" customWidth="1" min="30" max="30"/>
     <col width="16" customWidth="1" min="31" max="31"/>
     <col width="14" customWidth="1" min="32" max="32"/>
+    <col width="16" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1881,6 +1882,11 @@
       <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>sale_price</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>seller_email</t>
         </is>
       </c>
     </row>
@@ -1917,6 +1923,7 @@
       <c r="AD2" s="2" t="n"/>
       <c r="AE2" s="2" t="n"/>
       <c r="AF2" s="2" t="n"/>
+      <c r="AG2" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2470,12 +2477,12 @@
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -2530,12 +2537,12 @@
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -2594,12 +2601,12 @@
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -2658,12 +2665,12 @@
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -2718,12 +2725,12 @@
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -2778,12 +2785,12 @@
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -2838,12 +2845,12 @@
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -2898,12 +2905,12 @@
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -2958,12 +2965,12 @@
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -3018,12 +3025,12 @@
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -3078,12 +3085,12 @@
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -3138,12 +3145,12 @@
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -3198,12 +3205,12 @@
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -3258,12 +3265,12 @@
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="R15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -3318,12 +3325,12 @@
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="R16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -3378,12 +3385,12 @@
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="R17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -3438,12 +3445,12 @@
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="R18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -3498,12 +3505,12 @@
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -3558,12 +3565,12 @@
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="R20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -3618,12 +3625,12 @@
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="R21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -3678,12 +3685,12 @@
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="R22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -3738,12 +3745,12 @@
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
       <c r="R23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -3952,7 +3959,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -3974,7 +3981,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -3996,7 +4003,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -4018,7 +4025,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -4040,7 +4047,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4069,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -4074,7 +4081,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>1.4.0</t>
+          <t>1.5.0</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -4084,7 +4091,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4113,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -4128,7 +4135,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -4150,7 +4157,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4179,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:03:53.000Z</t>
+          <t>2026-09-12T17:37:10.000Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v1.6.0: Tools page reworked, and a way to empty the seeded inventory
Adding a build meant scrolling past every build already logged. The form is
now a single row of four fields at the top of the page, the inventory is two
columns, and the repeated status column is gone from the row. Date asked under
'Who hands over what' is a date picker rather than free text.

ClearTools.gs empties the inventory so real builds can be entered from
scratch. previewClearTools lists what would go; clearTools takes a full
backup first and stops if that fails, then clears the inventory, training and
runs. Afterwards setupDatabase will not re-seed the examples. It is the one
place in the desk that deletes rather than archives, so it is admin only, the
backup is the undo, and its test lives in the Node fixture rather than the
in-code suite, which runs against production.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PD4vD51siFq5jYyNjR6B3w
</commit_message>
<xml_diff>
--- a/apps/acquisitions-desk/docs/THB_Acquisitions_Desk_Production_Database_TEMPLATE.xlsx
+++ b/apps/acquisitions-desk/docs/THB_Acquisitions_Desk_Production_Database_TEMPLATE.xlsx
@@ -534,12 +534,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -579,12 +579,12 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -624,12 +624,12 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -665,12 +665,12 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -706,12 +706,12 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -747,12 +747,12 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -788,12 +788,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -829,12 +829,12 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -870,12 +870,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -911,12 +911,12 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -952,12 +952,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -993,12 +993,12 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -1034,12 +1034,12 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -1075,12 +1075,12 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -1116,12 +1116,12 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -1157,12 +1157,12 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -1198,12 +1198,12 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -1239,12 +1239,12 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -1280,12 +1280,12 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -1321,12 +1321,12 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -1403,12 +1403,12 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -1444,12 +1444,12 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -2477,12 +2477,12 @@
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -2537,12 +2537,12 @@
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -2601,12 +2601,12 @@
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -2665,12 +2665,12 @@
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -2725,12 +2725,12 @@
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -2785,12 +2785,12 @@
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -2845,12 +2845,12 @@
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -2905,12 +2905,12 @@
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -2965,12 +2965,12 @@
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -3025,12 +3025,12 @@
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -3085,12 +3085,12 @@
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -3145,12 +3145,12 @@
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -3205,12 +3205,12 @@
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -3265,12 +3265,12 @@
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="R15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -3325,12 +3325,12 @@
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="R16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -3385,12 +3385,12 @@
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="R17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -3445,12 +3445,12 @@
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="R18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -3505,12 +3505,12 @@
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -3565,12 +3565,12 @@
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="R20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -3625,12 +3625,12 @@
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="R21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -3685,12 +3685,12 @@
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="R22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -3745,12 +3745,12 @@
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
       <c r="R23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -3959,7 +3959,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -3981,7 +3981,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -4003,7 +4003,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -4025,7 +4025,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -4047,7 +4047,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -4069,7 +4069,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -4081,7 +4081,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>1.5.0</t>
+          <t>1.6.0</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -4091,7 +4091,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -4113,7 +4113,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -4135,7 +4135,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -4157,7 +4157,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>
@@ -4179,7 +4179,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T17:37:10.000Z</t>
+          <t>2026-09-12T18:31:13.000Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v1.6.1: filter the tool inventory by type instead of by builder
Every build gets a Type of System, Automation or Reporting. The inventory
tabs are those three plus All, set on the Log a build form and changeable on
the tool. A build with no type yet gets its own tab so nothing hides, and that
tab disappears once everything is typed. The row leads with the type in place
of the builder, who is still on the tool and in the handover panel.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PD4vD51siFq5jYyNjR6B3w
</commit_message>
<xml_diff>
--- a/apps/acquisitions-desk/docs/THB_Acquisitions_Desk_Production_Database_TEMPLATE.xlsx
+++ b/apps/acquisitions-desk/docs/THB_Acquisitions_Desk_Production_Database_TEMPLATE.xlsx
@@ -534,12 +534,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -579,12 +579,12 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -624,12 +624,12 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -665,12 +665,12 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -706,12 +706,12 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -747,12 +747,12 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -788,12 +788,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -829,12 +829,12 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -870,12 +870,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -911,12 +911,12 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -952,12 +952,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -993,12 +993,12 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -1034,12 +1034,12 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -1075,12 +1075,12 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -1116,12 +1116,12 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -1157,12 +1157,12 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -1198,12 +1198,12 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -1239,12 +1239,12 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -1280,12 +1280,12 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -1321,12 +1321,12 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -1403,12 +1403,12 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -1444,12 +1444,12 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -2311,7 +2311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R23"/>
+  <dimension ref="A1:S23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2332,6 +2332,7 @@
     <col width="14" customWidth="1" min="16" max="16"/>
     <col width="14" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2425,6 +2426,11 @@
           <t>updated_at</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>tool_type</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -2477,14 +2483,15 @@
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
-        </is>
-      </c>
+          <t>2026-09-12T20:59:48.000Z</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -2537,14 +2544,15 @@
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
-        </is>
-      </c>
+          <t>2026-09-12T20:59:48.000Z</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2601,14 +2609,15 @@
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
-        </is>
-      </c>
+          <t>2026-09-12T20:59:48.000Z</t>
+        </is>
+      </c>
+      <c r="S4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2665,14 +2674,15 @@
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
-        </is>
-      </c>
+          <t>2026-09-12T20:59:48.000Z</t>
+        </is>
+      </c>
+      <c r="S5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2725,14 +2735,15 @@
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
-        </is>
-      </c>
+          <t>2026-09-12T20:59:48.000Z</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2785,14 +2796,15 @@
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
-        </is>
-      </c>
+          <t>2026-09-12T20:59:48.000Z</t>
+        </is>
+      </c>
+      <c r="S7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2845,14 +2857,15 @@
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
-        </is>
-      </c>
+          <t>2026-09-12T20:59:48.000Z</t>
+        </is>
+      </c>
+      <c r="S8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2905,14 +2918,15 @@
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
-        </is>
-      </c>
+          <t>2026-09-12T20:59:48.000Z</t>
+        </is>
+      </c>
+      <c r="S9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2965,14 +2979,15 @@
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
-        </is>
-      </c>
+          <t>2026-09-12T20:59:48.000Z</t>
+        </is>
+      </c>
+      <c r="S10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3025,14 +3040,15 @@
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
-        </is>
-      </c>
+          <t>2026-09-12T20:59:48.000Z</t>
+        </is>
+      </c>
+      <c r="S11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3085,14 +3101,15 @@
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
-        </is>
-      </c>
+          <t>2026-09-12T20:59:48.000Z</t>
+        </is>
+      </c>
+      <c r="S12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3145,14 +3162,15 @@
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
-        </is>
-      </c>
+          <t>2026-09-12T20:59:48.000Z</t>
+        </is>
+      </c>
+      <c r="S13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3205,14 +3223,15 @@
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
-        </is>
-      </c>
+          <t>2026-09-12T20:59:48.000Z</t>
+        </is>
+      </c>
+      <c r="S14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3265,14 +3284,15 @@
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="R15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
-        </is>
-      </c>
+          <t>2026-09-12T20:59:48.000Z</t>
+        </is>
+      </c>
+      <c r="S15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3325,14 +3345,15 @@
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="R16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
-        </is>
-      </c>
+          <t>2026-09-12T20:59:48.000Z</t>
+        </is>
+      </c>
+      <c r="S16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -3385,14 +3406,15 @@
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="R17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
-        </is>
-      </c>
+          <t>2026-09-12T20:59:48.000Z</t>
+        </is>
+      </c>
+      <c r="S17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3445,14 +3467,15 @@
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="R18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
-        </is>
-      </c>
+          <t>2026-09-12T20:59:48.000Z</t>
+        </is>
+      </c>
+      <c r="S18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3505,14 +3528,15 @@
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
-        </is>
-      </c>
+          <t>2026-09-12T20:59:48.000Z</t>
+        </is>
+      </c>
+      <c r="S19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3565,14 +3589,15 @@
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="R20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
-        </is>
-      </c>
+          <t>2026-09-12T20:59:48.000Z</t>
+        </is>
+      </c>
+      <c r="S20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3625,14 +3650,15 @@
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="R21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
-        </is>
-      </c>
+          <t>2026-09-12T20:59:48.000Z</t>
+        </is>
+      </c>
+      <c r="S21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3685,14 +3711,15 @@
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="R22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
-        </is>
-      </c>
+          <t>2026-09-12T20:59:48.000Z</t>
+        </is>
+      </c>
+      <c r="S22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3745,14 +3772,15 @@
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
       <c r="R23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
-        </is>
-      </c>
+          <t>2026-09-12T20:59:48.000Z</t>
+        </is>
+      </c>
+      <c r="S23" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3959,7 +3987,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -3981,7 +4009,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -4003,7 +4031,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -4025,7 +4053,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -4047,7 +4075,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -4069,7 +4097,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -4081,7 +4109,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>1.6.0</t>
+          <t>1.6.1</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -4091,7 +4119,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -4113,7 +4141,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -4135,7 +4163,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -4157,7 +4185,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>
@@ -4179,7 +4207,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T18:31:13.000Z</t>
+          <t>2026-09-12T20:59:48.000Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v1.7.0: split Wholesale into assignment and double close, and make the money follow
The desk assumed every deal is buy then sell. On an assignment we never own
the house, so subtracting a purchase from a fee produced a large fake loss.

Wholesale is now two exit strategies. An assignment labels the purchase price
as the contract price, replaces sale price with an assignment fee, and treats
the fee as what we make. Every other exit keeps both prices and the existing
profit maths. The board row follows the same rule.

Two guards where the typo hides: a sale price on an assignment is flagged with
a note to move it to the fee, and a sale below the purchase on any other exit
is flagged as a real loss unless a number is wrong. Records written before the
split keep the plain Wholesale value, which stays savable and appears in the
dropdown on those records only.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PD4vD51siFq5jYyNjR6B3w
</commit_message>
<xml_diff>
--- a/apps/acquisitions-desk/docs/THB_Acquisitions_Desk_Production_Database_TEMPLATE.xlsx
+++ b/apps/acquisitions-desk/docs/THB_Acquisitions_Desk_Production_Database_TEMPLATE.xlsx
@@ -534,12 +534,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -579,12 +579,12 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -624,12 +624,12 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -665,12 +665,12 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -706,12 +706,12 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -747,12 +747,12 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -788,12 +788,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -829,12 +829,12 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -870,12 +870,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -911,12 +911,12 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -952,12 +952,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -993,12 +993,12 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -1034,12 +1034,12 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -1075,12 +1075,12 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -1116,12 +1116,12 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -1157,12 +1157,12 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -1198,12 +1198,12 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -1239,12 +1239,12 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -1280,12 +1280,12 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -1321,12 +1321,12 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -1403,12 +1403,12 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -1444,12 +1444,12 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -1685,7 +1685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG2"/>
+  <dimension ref="A1:AH2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1721,6 +1721,7 @@
     <col width="16" customWidth="1" min="31" max="31"/>
     <col width="14" customWidth="1" min="32" max="32"/>
     <col width="16" customWidth="1" min="33" max="33"/>
+    <col width="18" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1887,6 +1888,11 @@
       <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>seller_email</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>assignment_fee</t>
         </is>
       </c>
     </row>
@@ -1924,6 +1930,7 @@
       <c r="AE2" s="2" t="n"/>
       <c r="AF2" s="2" t="n"/>
       <c r="AG2" s="2" t="n"/>
+      <c r="AH2" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2483,12 +2490,12 @@
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="S2" s="2" t="n"/>
@@ -2544,12 +2551,12 @@
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="S3" s="2" t="n"/>
@@ -2609,12 +2616,12 @@
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="S4" s="2" t="n"/>
@@ -2674,12 +2681,12 @@
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="S5" s="2" t="n"/>
@@ -2735,12 +2742,12 @@
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="S6" s="2" t="n"/>
@@ -2796,12 +2803,12 @@
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="S7" s="2" t="n"/>
@@ -2857,12 +2864,12 @@
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="S8" s="2" t="n"/>
@@ -2918,12 +2925,12 @@
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="S9" s="2" t="n"/>
@@ -2979,12 +2986,12 @@
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="S10" s="2" t="n"/>
@@ -3040,12 +3047,12 @@
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="S11" s="2" t="n"/>
@@ -3101,12 +3108,12 @@
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="S12" s="2" t="n"/>
@@ -3162,12 +3169,12 @@
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="S13" s="2" t="n"/>
@@ -3223,12 +3230,12 @@
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="S14" s="2" t="n"/>
@@ -3284,12 +3291,12 @@
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="R15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="S15" s="2" t="n"/>
@@ -3345,12 +3352,12 @@
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="R16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="S16" s="2" t="n"/>
@@ -3406,12 +3413,12 @@
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="R17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="S17" s="2" t="n"/>
@@ -3467,12 +3474,12 @@
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="R18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="S18" s="2" t="n"/>
@@ -3528,12 +3535,12 @@
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="S19" s="2" t="n"/>
@@ -3589,12 +3596,12 @@
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="R20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="S20" s="2" t="n"/>
@@ -3650,12 +3657,12 @@
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="R21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="S21" s="2" t="n"/>
@@ -3711,12 +3718,12 @@
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="R22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="S22" s="2" t="n"/>
@@ -3772,12 +3779,12 @@
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="R23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
       <c r="S23" s="2" t="n"/>
@@ -3987,7 +3994,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -4009,7 +4016,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -4031,7 +4038,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -4053,7 +4060,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -4075,7 +4082,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -4097,7 +4104,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -4109,7 +4116,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>1.6.1</t>
+          <t>1.7.0</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -4119,7 +4126,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -4141,7 +4148,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -4163,7 +4170,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -4185,7 +4192,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>
@@ -4207,7 +4214,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12T20:59:48.000Z</t>
+          <t>2026-09-12T22:20:23.000Z</t>
         </is>
       </c>
     </row>

</xml_diff>